<commit_message>
docs: align case timeline with August 10 kickoff
</commit_message>
<xml_diff>
--- a/Task2/tco-model.xlsx
+++ b/Task2/tco-model.xlsx
@@ -12418,15 +12418,17 @@
       <x:c r="G34" s="55"/>
       <x:c r="H34" s="55"/>
     </x:row>
-    <x:row r="35" ht="48" customHeight="1">
+    <x:row r="35" ht="58" customHeight="1">
       <x:c r="B35" s="55" t="str">
         <x:v>USD за Processor Oracle EE</x:v>
       </x:c>
       <x:c r="C35" s="173" t="n">
         <x:v>47500</x:v>
       </x:c>
-      <x:c r="D35" s="55" t="str">
-        <x:v>Публичный Oracle Price List 15.09.2026, с.2; не скидка/оферта, метрика Processor не vCPU.</x:v>
+      <x:c r="D35" s="55" t="inlineStr">
+        <x:is>
+          <x:t>Oracle Price List 15.09.2026, с.2 — позднее уточнение, не источник, известный 10.08. Для первоначального выбора цена оценочная до раннего прайса/оферты. Processor не vCPU.</x:t>
+        </x:is>
       </x:c>
       <x:c r="E35" s="55"/>
       <x:c r="F35" s="55"/>
@@ -13624,9 +13626,11 @@
       <x:c r="G135" s="55"/>
       <x:c r="H135" s="55"/>
     </x:row>
-    <x:row r="136" ht="36" customHeight="1">
-      <x:c r="B136" s="180" t="str">
-        <x:v>Источники цен проверены 05.10.2026. Публичные тарифы не заменяют локальную оферту / лицензионный расчёт.</x:v>
+    <x:row r="136" ht="48" customHeight="1">
+      <x:c r="B136" s="180" t="inlineStr">
+        <x:is>
+          <x:t>Фактическая проверка цен: 05.10.2026, позднее начала кейса 10.08. Для августовского выбора цены — плановые допущения до исторической редакции или оферты; дата проверки не переносится на август.</x:t>
+        </x:is>
       </x:c>
       <x:c r="C136" s="180"/>
       <x:c r="D136" s="180"/>
@@ -13719,9 +13723,11 @@
       <x:c r="G144" s="55"/>
       <x:c r="H144" s="55"/>
     </x:row>
-    <x:row r="145" ht="35" customHeight="1">
-      <x:c r="B145" s="55" t="str">
-        <x:v>Календарь: сегодня 05.10.2026, встреча 12.10, запуск 15.10. Оценки 8/12/24 недели — от готовой команды и договоров. При старте с нуля сейчас ни один полный MVP не успеет; готовность неизвестна.</x:v>
+    <x:row r="145" ht="52" customHeight="1">
+      <x:c r="B145" s="55" t="inlineStr">
+        <x:is>
+          <x:t>Кейс: начало 10.08.2026, встреча ориентир 17.08, открытие 15.10. A (8 недель) готов 05.10: резерв 10 дней; B (12 недель) 02.11: +18 дней; C (24 недели) 25.01.2027: +102 дня. Старт работ 10.08 условен: нужна готовая команда. Дата проверки цен не меняет календарь.</x:t>
+        </x:is>
       </x:c>
       <x:c r="C145" s="55"/>
       <x:c r="D145" s="55"/>

</xml_diff>